<commit_message>
CoA: Schedule III order + correct CGST/SGST half-slab naming; regenerate all outputs
</commit_message>
<xml_diff>
--- a/output/gstr2b_recon_truth.xlsx
+++ b/output/gstr2b_recon_truth.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recon Truth" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Recon Truth" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <name val="Tahoma"/>
@@ -62,19 +59,13 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
     </border>
     <border>
       <left style="thin">
@@ -96,20 +87,20 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>